<commit_message>
fixing to correct version of UDAQ mapping to mechanisms
</commit_message>
<xml_diff>
--- a/Hawthorne_data/EPA_CRACMM_GEOSCHEM_mapped.xlsx
+++ b/Hawthorne_data/EPA_CRACMM_GEOSCHEM_mapped.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u1545774\Documents\GitHub\USOS_shared\Hawthorne_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u1545774\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{8EA3D69A-6705-49EE-98C4-DFBC8364BF15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A994259A-FAA4-469C-9734-026AFA7C8458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1935" yWindow="52" windowWidth="27098" windowHeight="8715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EPA_CRACMM_GEOSCHEM_mapped" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="540">
   <si>
     <t>Parameter Code</t>
   </si>
@@ -1642,6 +1642,9 @@
   </si>
   <si>
     <t>Styrene_PTR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">probably TMB, but ask Kelvin </t>
   </si>
 </sst>
 </file>
@@ -1709,7 +1712,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1754,7 +1757,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1764,10 +1767,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2071,16 +2075,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V61"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.46484375" customWidth="1"/>
-    <col min="19" max="19" width="18.86328125" customWidth="1"/>
-    <col min="20" max="20" width="20.19921875" customWidth="1"/>
-    <col min="21" max="21" width="16.73046875" customWidth="1"/>
-    <col min="22" max="22" width="22.59765625" customWidth="1"/>
+    <col min="1" max="1" width="29.33203125" customWidth="1"/>
+    <col min="2" max="2" width="37.109375" customWidth="1"/>
+    <col min="4" max="4" width="22.5546875" customWidth="1"/>
+    <col min="5" max="5" width="29.33203125" customWidth="1"/>
+    <col min="19" max="19" width="18.88671875" customWidth="1"/>
+    <col min="20" max="20" width="20.21875" customWidth="1"/>
+    <col min="21" max="21" width="16.77734375" customWidth="1"/>
+    <col min="22" max="22" width="22.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2141,14 +2148,14 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="U1" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="V1" s="6" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>43102</v>
       </c>
@@ -2168,7 +2175,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>43141</v>
       </c>
@@ -2227,7 +2234,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>43202</v>
       </c>
@@ -2288,14 +2295,14 @@
       <c r="T4" t="s">
         <v>37</v>
       </c>
-      <c r="U4" s="6" t="s">
+      <c r="U4" s="5" t="s">
         <v>514</v>
       </c>
       <c r="V4" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>43203</v>
       </c>
@@ -2363,7 +2370,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>43204</v>
       </c>
@@ -2424,14 +2431,14 @@
       <c r="T6" t="s">
         <v>55</v>
       </c>
-      <c r="U6" s="6" t="s">
+      <c r="U6" s="5" t="s">
         <v>515</v>
       </c>
       <c r="V6" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>43205</v>
       </c>
@@ -2496,7 +2503,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>43206</v>
       </c>
@@ -2560,11 +2567,11 @@
       <c r="U8" t="s">
         <v>516</v>
       </c>
-      <c r="V8" s="8" t="s">
+      <c r="V8" s="7" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>43212</v>
       </c>
@@ -2629,7 +2636,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>43214</v>
       </c>
@@ -2687,14 +2694,14 @@
       <c r="S10" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="T10" s="5" t="s">
+      <c r="T10" s="8" t="s">
         <v>91</v>
       </c>
       <c r="V10" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>43216</v>
       </c>
@@ -2752,8 +2759,11 @@
       <c r="S11" s="4" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>43217</v>
       </c>
@@ -2811,8 +2821,11 @@
       <c r="S12" s="4" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>43218</v>
       </c>
@@ -2874,7 +2887,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>43220</v>
       </c>
@@ -2932,14 +2945,14 @@
       <c r="S14" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="T14" s="5" t="s">
+      <c r="T14" s="9" t="s">
         <v>91</v>
       </c>
       <c r="V14" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>43221</v>
       </c>
@@ -2997,11 +3010,11 @@
       <c r="S15" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="T15" s="5" t="s">
+      <c r="T15" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>43224</v>
       </c>
@@ -3059,8 +3072,11 @@
       <c r="S16" s="4" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T16" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>43226</v>
       </c>
@@ -3118,8 +3134,11 @@
       <c r="S17" s="4" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T17" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>43227</v>
       </c>
@@ -3177,8 +3196,11 @@
       <c r="S18" s="4" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T18" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>43230</v>
       </c>
@@ -3236,11 +3258,11 @@
       <c r="S19" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="T19" s="5" t="s">
+      <c r="T19" s="9" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>43231</v>
       </c>
@@ -3298,14 +3320,14 @@
       <c r="S20" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="T20" s="5" t="s">
+      <c r="T20" s="9" t="s">
         <v>512</v>
       </c>
       <c r="V20" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>43232</v>
       </c>
@@ -3363,11 +3385,14 @@
       <c r="S21" s="3" t="s">
         <v>191</v>
       </c>
+      <c r="T21" t="s">
+        <v>512</v>
+      </c>
       <c r="V21" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>43233</v>
       </c>
@@ -3425,11 +3450,14 @@
       <c r="S22" s="3" t="s">
         <v>191</v>
       </c>
+      <c r="T22" t="s">
+        <v>512</v>
+      </c>
       <c r="V22" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>43235</v>
       </c>
@@ -3487,11 +3515,14 @@
       <c r="S23" s="3" t="s">
         <v>191</v>
       </c>
+      <c r="T23" t="s">
+        <v>512</v>
+      </c>
       <c r="V23" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>43238</v>
       </c>
@@ -3549,8 +3580,11 @@
       <c r="S24" s="4" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T24" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>43242</v>
       </c>
@@ -3608,11 +3642,11 @@
       <c r="S25" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="T25" s="5" t="s">
+      <c r="T25" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>43243</v>
       </c>
@@ -3680,7 +3714,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>43244</v>
       </c>
@@ -3738,11 +3772,11 @@
       <c r="S27" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="T27" s="5" t="s">
+      <c r="T27" s="9" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>43245</v>
       </c>
@@ -3800,11 +3834,11 @@
       <c r="S28" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="T28" s="5" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T28" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>43247</v>
       </c>
@@ -3862,8 +3896,11 @@
       <c r="S29" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T29" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>43248</v>
       </c>
@@ -3921,11 +3958,11 @@
       <c r="S30" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="T30" s="5" t="s">
+      <c r="T30" s="9" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>43249</v>
       </c>
@@ -3983,8 +4020,11 @@
       <c r="S31" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T31" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>43250</v>
       </c>
@@ -4042,8 +4082,11 @@
       <c r="S32" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T32" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>43252</v>
       </c>
@@ -4101,8 +4144,11 @@
       <c r="S33" s="3" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T33" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>43253</v>
       </c>
@@ -4160,8 +4206,11 @@
       <c r="S34" s="3" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T34" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>43261</v>
       </c>
@@ -4219,8 +4268,11 @@
       <c r="S35" s="3" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T35" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>43262</v>
       </c>
@@ -4278,11 +4330,11 @@
       <c r="S36" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="T36" s="5" t="s">
+      <c r="T36" s="9" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>43263</v>
       </c>
@@ -4340,8 +4392,11 @@
       <c r="S37" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T37" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>43280</v>
       </c>
@@ -4399,8 +4454,11 @@
       <c r="S38" s="4" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T38" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>43284</v>
       </c>
@@ -4458,11 +4516,11 @@
       <c r="S39" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="T39" s="5" t="s">
+      <c r="T39" s="9" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>43285</v>
       </c>
@@ -4520,11 +4578,11 @@
       <c r="S40" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="T40" s="5" t="s">
+      <c r="T40" s="9" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>43291</v>
       </c>
@@ -4582,8 +4640,11 @@
       <c r="S41" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T41" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>43502</v>
       </c>
@@ -4648,7 +4709,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>43954</v>
       </c>
@@ -4706,8 +4767,11 @@
       <c r="S43" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T43" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43960</v>
       </c>
@@ -4765,8 +4829,11 @@
       <c r="S44" s="3" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T44" s="9" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>45109</v>
       </c>
@@ -4821,7 +4888,7 @@
       <c r="S45" t="s">
         <v>377</v>
       </c>
-      <c r="T45" s="5" t="s">
+      <c r="T45" s="9" t="s">
         <v>509</v>
       </c>
       <c r="U45" t="s">
@@ -4831,7 +4898,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45109</v>
       </c>
@@ -4886,7 +4953,7 @@
       <c r="S46" t="s">
         <v>377</v>
       </c>
-      <c r="T46" s="5" t="s">
+      <c r="T46" s="9" t="s">
         <v>509</v>
       </c>
       <c r="U46" t="s">
@@ -4896,7 +4963,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>45201</v>
       </c>
@@ -4954,7 +5021,7 @@
       <c r="S47" t="s">
         <v>392</v>
       </c>
-      <c r="T47" t="s">
+      <c r="T47" s="9" t="s">
         <v>393</v>
       </c>
       <c r="U47" t="s">
@@ -4964,7 +5031,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>45202</v>
       </c>
@@ -5022,7 +5089,7 @@
       <c r="S48" t="s">
         <v>402</v>
       </c>
-      <c r="T48" t="s">
+      <c r="T48" s="9" t="s">
         <v>403</v>
       </c>
       <c r="U48" t="s">
@@ -5032,7 +5099,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>45203</v>
       </c>
@@ -5090,7 +5157,7 @@
       <c r="S49" t="s">
         <v>411</v>
       </c>
-      <c r="T49" t="s">
+      <c r="T49" s="9" t="s">
         <v>411</v>
       </c>
       <c r="U49" t="s">
@@ -5100,7 +5167,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>45204</v>
       </c>
@@ -5158,14 +5225,14 @@
       <c r="S50" t="s">
         <v>377</v>
       </c>
-      <c r="T50" s="5" t="s">
+      <c r="T50" s="9" t="s">
         <v>509</v>
       </c>
       <c r="V50" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>45207</v>
       </c>
@@ -5227,7 +5294,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>45208</v>
       </c>
@@ -5289,7 +5356,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>45209</v>
       </c>
@@ -5347,8 +5414,11 @@
       <c r="S53" s="3" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T53" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>45210</v>
       </c>
@@ -5406,8 +5476,11 @@
       <c r="S54" s="3" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T54" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>45211</v>
       </c>
@@ -5465,8 +5538,11 @@
       <c r="S55" s="3" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T55" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>45212</v>
       </c>
@@ -5524,8 +5600,11 @@
       <c r="S56" s="3" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T56" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>45213</v>
       </c>
@@ -5583,8 +5662,11 @@
       <c r="S57" s="3" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T57" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>45218</v>
       </c>
@@ -5642,8 +5724,11 @@
       <c r="S58" s="3" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T58" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>45219</v>
       </c>
@@ -5701,11 +5786,14 @@
       <c r="S59" s="3" t="s">
         <v>377</v>
       </c>
+      <c r="T59" t="s">
+        <v>539</v>
+      </c>
       <c r="V59" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>45220</v>
       </c>
@@ -5767,7 +5855,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>45225</v>
       </c>

</xml_diff>